<commit_message>
FIXUAE-211 Replaced template file Import Abonents with a new one
</commit_message>
<xml_diff>
--- a/assets/abonent-import-template_ru.xlsx
+++ b/assets/abonent-import-template_ru.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Vladimir\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nosleep\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{64704DD7-773F-4A1C-AE24-81EC51AAE4AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="18045" windowHeight="11325"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>ФИО</t>
   </si>
@@ -62,11 +63,14 @@
   <si>
     <t>Код rfid метки для парковок</t>
   </si>
+  <si>
+    <t>Лицевой счет</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -146,7 +150,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -168,9 +172,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -206,7 +207,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Рисунок 1"/>
+        <xdr:cNvPr id="2" name="Рисунок 1">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -244,7 +251,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="7" name="Рисунок 6"/>
+        <xdr:cNvPr id="7" name="Рисунок 6">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000007000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -281,7 +294,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="8" name="Рисунок 7"/>
+        <xdr:cNvPr id="8" name="Рисунок 7">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000008000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -319,7 +338,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="9" name="Рисунок 8"/>
+        <xdr:cNvPr id="9" name="Рисунок 8">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000009000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -357,7 +382,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="12" name="Рисунок 11"/>
+        <xdr:cNvPr id="12" name="Рисунок 11">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-00000C000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -395,7 +426,13 @@
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Рисунок 3"/>
+        <xdr:cNvPr id="4" name="Рисунок 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000004000000}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -682,7 +719,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:N39"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
@@ -1317,7 +1354,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AA2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -1371,7 +1408,9 @@
       <c r="L1" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="M1" s="8"/>
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
       <c r="N1" s="7"/>
       <c r="O1" s="7"/>
       <c r="P1" s="7"/>

</xml_diff>